<commit_message>
Update Path 2 brand quiz high-res images, fix MBA-BQ-2 code, remove redundant QR completion code, and refine word search flow
</commit_message>
<xml_diff>
--- a/ROUTE_1_PATH1_ECE_MECH_FC_CY_AUDI/PATH1_FINAL_ODK.xlsx
+++ b/ROUTE_1_PATH1_ECE_MECH_FC_CY_AUDI/PATH1_FINAL_ODK.xlsx
@@ -483,7 +483,8 @@
 • Round 3 ➔ Round 4: Next 7 teams proceed
 • Round 4 ➔ Round 5: Next 2 teams proceed
 from each path
-⚠️ MANDATORY RESPONSE &amp; CAPS ONLY RULES:
+⚠️ STRICT PROGRESSION &amp; MANDATORY RULES:
+• Read each question properly as you cannot come back to the question once you go ahead!
 • Every single question and upload is strictly MANDATORY.
 • All text answers and volunteer clearance codes must be entered in UPPERCASE (CAPS ONLY).
 • Lowercase letters will be rejected.</v>
@@ -504,7 +505,7 @@
 Enter code in caps</v>
       </c>
       <c r="D4" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E4" t="str">
         <v>yes</v>
@@ -531,7 +532,7 @@
 Enter in caps</v>
       </c>
       <c r="D5" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E5" t="str">
         <v>yes</v>
@@ -615,7 +616,7 @@
 Enter code in caps</v>
       </c>
       <c r="D10" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E10" t="str">
         <v>yes</v>
@@ -679,7 +680,7 @@
 Enter code in caps</v>
       </c>
       <c r="D14" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E14" t="str">
         <v>yes</v>
@@ -725,7 +726,7 @@
 Enter code in caps</v>
       </c>
       <c r="D16" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E16" t="str">
         <v>yes</v>
@@ -913,7 +914,7 @@
 Enter code in caps</v>
       </c>
       <c r="D26" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E26" t="str">
         <v>yes</v>
@@ -978,7 +979,7 @@
 Enter code in caps</v>
       </c>
       <c r="D30" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E30" t="str">
         <v>yes</v>
@@ -1050,7 +1051,7 @@
 Enter code in caps</v>
       </c>
       <c r="D35" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E35" t="str">
         <v>yes</v>
@@ -1077,7 +1078,7 @@
 Enter code in caps</v>
       </c>
       <c r="D36" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E36" t="str">
         <v>yes</v>
@@ -1104,7 +1105,7 @@
 Enter code in caps</v>
       </c>
       <c r="D37" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E37" t="str">
         <v>yes</v>
@@ -1131,7 +1132,7 @@
 Enter code in caps</v>
       </c>
       <c r="D38" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E38" t="str">
         <v>yes</v>
@@ -1158,7 +1159,7 @@
 Enter code in caps</v>
       </c>
       <c r="D39" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E39" t="str">
         <v>yes</v>
@@ -1191,7 +1192,7 @@
 Enter code in caps</v>
       </c>
       <c r="D40" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E40" t="str">
         <v>yes</v>
@@ -1283,7 +1284,7 @@
 Enter code in caps</v>
       </c>
       <c r="D45" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E45" t="str">
         <v>yes</v>
@@ -1355,7 +1356,7 @@
 Enter code in caps</v>
       </c>
       <c r="D49" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E49" t="str">
         <v>yes</v>
@@ -1418,7 +1419,7 @@
 Enter code in caps</v>
       </c>
       <c r="D53" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E53" t="str">
         <v>yes</v>
@@ -1464,7 +1465,7 @@
 Enter code in caps</v>
       </c>
       <c r="D55" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E55" t="str">
         <v>yes</v>
@@ -1535,7 +1536,7 @@
 Enter code in caps</v>
       </c>
       <c r="D59" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E59" t="str">
         <v>yes</v>
@@ -1563,7 +1564,7 @@
 Enter code in caps</v>
       </c>
       <c r="D60" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E60" t="str">
         <v>yes</v>
@@ -1637,7 +1638,7 @@
 Enter code in caps</v>
       </c>
       <c r="D63" t="str">
-        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY.</v>
+        <v>ENTER CODE/ANSWER IN CAPITAL LETTERS ONLY. Read the question properly as you cannot come back to the question once you go ahead.</v>
       </c>
       <c r="E63" t="str">
         <v>yes</v>

</xml_diff>